<commit_message>
ajout de plus d'animation dans la page d'accueil
</commit_message>
<xml_diff>
--- a/assets/CV/Tableau_de_synthese_Ouss.xlsx
+++ b/assets/CV/Tableau_de_synthese_Ouss.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ousse\Desktop\portfolio\assets\CV\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E42527CD-4CDA-4635-A999-B192F6CFBB40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2079BD94-904F-4F58-8FEB-7553F6BBC5FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="45">
   <si>
     <t>BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
   </si>
@@ -164,10 +164,19 @@
     <t>Aide support au utilisateurs</t>
   </si>
   <si>
-    <t xml:space="preserve">Masterisation de Poste Via PXE boot </t>
-  </si>
-  <si>
-    <t>Gestion de ticket via GLPI</t>
+    <t>Aide et support aux utilisateurs (incidents postes, écrans, logiciels, demandes diverses)</t>
+  </si>
+  <si>
+    <t>Masterisation et déploiement de postes Lenovo (E15, E16, L14) via PXE boot</t>
+  </si>
+  <si>
+    <t>Préparation et configuration de smartphones professionnels (Samsung Galaxy A16)</t>
+  </si>
+  <si>
+    <t>Gestion des tickets d’incidents et de demandes via GLPI</t>
+  </si>
+  <si>
+    <t>Gestion de parc et des comptes via Active Directory (création/modification/ désactivation, ajout de postes au domaine)</t>
   </si>
 </sst>
 </file>
@@ -177,7 +186,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$€-1]_-;\-* #,##0.00\ [$€-1]_-;_-* &quot;-&quot;??\ [$€-1]_-"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color theme="1"/>
@@ -236,6 +245,12 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -664,7 +679,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -811,6 +826,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2295,10 +2316,14 @@
       </c>
       <c r="B28" s="48"/>
       <c r="C28" s="13"/>
-      <c r="D28" s="13"/>
+      <c r="D28" s="49" t="s">
+        <v>24</v>
+      </c>
       <c r="E28" s="13"/>
       <c r="F28" s="13"/>
-      <c r="G28" s="13"/>
+      <c r="G28" s="49" t="s">
+        <v>24</v>
+      </c>
       <c r="H28" s="14"/>
       <c r="I28"/>
       <c r="J28"/>
@@ -2341,7 +2366,9 @@
         <v>40</v>
       </c>
       <c r="B29" s="11"/>
-      <c r="C29" s="13"/>
+      <c r="C29" s="49" t="s">
+        <v>24</v>
+      </c>
       <c r="D29" s="13"/>
       <c r="E29" s="13"/>
       <c r="F29" s="13"/>
@@ -2386,11 +2413,13 @@
       <c r="AQ29"/>
     </row>
     <row r="30" spans="1:43" s="7" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="10" t="s">
+      <c r="A30" s="50" t="s">
         <v>41</v>
       </c>
       <c r="B30" s="11"/>
-      <c r="C30" s="13"/>
+      <c r="C30" s="49" t="s">
+        <v>24</v>
+      </c>
       <c r="D30" s="13"/>
       <c r="E30" s="13"/>
       <c r="F30" s="13"/>
@@ -2435,13 +2464,19 @@
       <c r="AQ30"/>
     </row>
     <row r="31" spans="1:43" s="7" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="10"/>
+      <c r="A31" s="50" t="s">
+        <v>42</v>
+      </c>
       <c r="B31" s="11"/>
-      <c r="C31" s="13"/>
+      <c r="C31" s="49" t="s">
+        <v>24</v>
+      </c>
       <c r="D31" s="13"/>
       <c r="E31" s="13"/>
       <c r="F31" s="13"/>
-      <c r="G31" s="13"/>
+      <c r="G31" s="49" t="s">
+        <v>24</v>
+      </c>
       <c r="H31" s="14"/>
       <c r="I31"/>
       <c r="J31"/>
@@ -2480,13 +2515,19 @@
       <c r="AQ31"/>
     </row>
     <row r="32" spans="1:43" s="7" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="10"/>
+      <c r="A32" s="10" t="s">
+        <v>43</v>
+      </c>
       <c r="B32" s="11"/>
       <c r="C32" s="13"/>
-      <c r="D32" s="13"/>
+      <c r="D32" s="49" t="s">
+        <v>24</v>
+      </c>
       <c r="E32" s="13"/>
       <c r="F32" s="13"/>
-      <c r="G32" s="13"/>
+      <c r="G32" s="49" t="s">
+        <v>24</v>
+      </c>
       <c r="H32" s="14"/>
       <c r="I32"/>
       <c r="J32"/>
@@ -2525,14 +2566,20 @@
       <c r="AQ32"/>
     </row>
     <row r="33" spans="1:43" s="7" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="10"/>
+      <c r="A33" s="10" t="s">
+        <v>44</v>
+      </c>
       <c r="B33" s="11"/>
-      <c r="C33" s="13"/>
+      <c r="C33" s="49" t="s">
+        <v>24</v>
+      </c>
       <c r="D33" s="13"/>
       <c r="E33" s="13"/>
       <c r="F33" s="13"/>
       <c r="G33" s="13"/>
-      <c r="H33" s="14"/>
+      <c r="H33" s="51" t="s">
+        <v>24</v>
+      </c>
       <c r="I33"/>
       <c r="J33"/>
       <c r="K33"/>
@@ -2569,7 +2616,7 @@
       <c r="AP33"/>
       <c r="AQ33"/>
     </row>
-    <row r="34" spans="1:43" s="7" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:43" s="7" customFormat="1" ht="39.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="19"/>
       <c r="B34" s="20"/>
       <c r="C34" s="21"/>

</xml_diff>